<commit_message>
docs: correct claims, document new behaviour; release 0.2.0
Bounded-memory, read-only, dialect, and export-parity wording now
matches tested behaviour. New parameters/timezone/currency/dry-run/
manifest/data-quality documentation; samples regenerated.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/examples/reports/sales-report-sample.xlsx
+++ b/examples/reports/sales-report-sample.xlsx
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -548,7 +548,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-28 20:11 UTC</t>
+          <t>2026-10-30 18:47 UTC</t>
         </is>
       </c>
     </row>
@@ -704,20 +704,35 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
+          <t>Methodology</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Revenue is taken from the source file (quantity × unit price at order time). Monthly figures group orders by calendar month of the order date.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
           <t>Sources</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
+    <row r="23">
+      <c r="A23" t="inlineStr">
         <is>
           <t>sales: CSV file synthetic_sales.csv (818 rows)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A9:D9"/>
+    <mergeCell ref="A20:D20"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>